<commit_message>
data: merge August channel backfill
</commit_message>
<xml_diff>
--- a/channel-maintenance-pv-fixed.xlsx
+++ b/channel-maintenance-pv-fixed.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R820b939a5eca4927"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="定义与优先级" sheetId="2" r:id="Rd90e77903c6b4589"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题清单" sheetId="3" r:id="R11a5b2b35f4f4a8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周采集明细" sheetId="4" r:id="Rc9ea382f7b7a43ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="渠道维护总表" sheetId="5" r:id="R8872721c025a465d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="Rb14bb4c440164193"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="定义与优先级" sheetId="2" r:id="Rb90fe51ca2bb429e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题清单" sheetId="3" r:id="Ra313d2d4024c49d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周采集明细" sheetId="4" r:id="R09efb064357149b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="渠道维护总表" sheetId="5" r:id="R138856ad05704577"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3827,7 +3827,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58cd2fbe55874da3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8231e6c89bc7439f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4298,7 +4298,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8aa99804c04f4724"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R009bad2da34f4077"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4631,7 +4631,7 @@
         <x:v>2026-08-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="132" customHeight="1">
+    <x:row r="5" ht="186" customHeight="1">
       <x:c r="A5" s="82" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -4702,13 +4702,15 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="X5" s="70" t="str">
-        <x:v>更新 sources.xlsx RSS 配置；新增源站 RSS 链接过滤钩子；回补 2026-07-29—2026-08-04 可用日期。</x:v>
+        <x:v>更新 sources.xlsx RSS 配置；新增源站 RSS 链接过滤钩子；回补 2026-07-29—2026-08-04 可用日期。
+2026-08-06 历史数据合并：08-04发布记录8条按规范化URL去重并新增，重新生成对应CSV。</x:v>
       </x:c>
       <x:c r="Y5" s="70" t="str">
-        <x:v>验证通过：07-29 4篇、07-30 3篇、07-31 4篇、08-04 8篇，合计19篇；URL唯一19，正文可用19篇；08-04状态 healthy。</x:v>
+        <x:v>验证通过：07-29 4篇、07-30 3篇、07-31 4篇、08-04 8篇，合计19篇；URL唯一19，正文可用19篇；08-04状态 healthy。
+新增8条、重复0条；正文376—1,674字，8条均通过完整性检查。</x:v>
       </x:c>
       <x:c r="Z5" s="70" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>2026-08-06</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -4925,7 +4927,7 @@
         <x:v>2026-08-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="156" customHeight="1">
+    <x:row r="9" ht="186" customHeight="1">
       <x:c r="A9" s="82" t="n">
         <x:v>8</x:v>
       </x:c>
@@ -4992,13 +4994,14 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="X9" s="70" t="str">
-        <x:v>新增 InterestingEngineeringScraper、分页和时区测试；主流程支持定制抓取器自行组合已配置RSS；正文选择器限定 .body-content。</x:v>
+        <x:v>新增 InterestingEngineeringScraper、分页和时区测试；主流程支持定制抓取器自行组合已配置RSS；正文选择器限定 .body-content。
+新增分页、时区、RSS全文优先与公开预览边界测试；主流程支持定制抓取器组合已配置RSS；public_preview 纳入 incomplete/degraded 质量口径。</x:v>
       </x:c>
       <x:c r="Y9" s="70" t="str">
-        <x:v>新增分页、时区、RSS全文优先与公开预览边界测试；主流程支持定制抓取器组合已配置RSS；public_preview 纳入 incomplete/degraded 质量口径。</x:v>
+        <x:v>链路回测两日共采集33篇且URL唯一；RSS content:encoded 命中项可验证为全文，未命中项只保留公开预览并明确降级，不能再按旧字数阈值宣称33篇均为全文。</x:v>
       </x:c>
       <x:c r="Z9" s="70" t="str">
-        <x:v>链路回测两日共采集33篇且URL唯一；RSS content:encoded 命中项可验证为全文，未命中项只保留公开预览并明确降级，不能再按旧字数阈值宣称33篇均为全文。</x:v>
+        <x:v>2026-08-06</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -5361,7 +5364,7 @@
         <x:v>2026-08-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="158" customHeight="1">
+    <x:row r="15" ht="186" customHeight="1">
       <x:c r="A15" s="82" t="n">
         <x:v>14</x:v>
       </x:c>
@@ -5432,13 +5435,15 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="X15" s="70" t="str">
-        <x:v>2026-08-05 实网测试 latest-news 列表、Next 分页及详情正文均正常；正式回补 2026-08-01—08-05，写入 data/articles.jsonl 和逐日 CSV。</x:v>
+        <x:v>2026-08-05 实网测试 latest-news 列表、Next 分页及详情正文均正常；正式回补 2026-08-01—08-05，写入 data/articles.jsonl 和逐日 CSV。
+2026-08-06 历史数据合并：筛选08-01—08-05发布记录19条，按全库规范化URL去重后新增4条，远端已存在15条；重新生成08-03、08-04发布日对应CSV。</x:v>
       </x:c>
       <x:c r="Y15" s="70" t="str">
-        <x:v>验证通过：08-01 idle 0；08-02 idle 0；08-03 13；08-04 6；08-05 0（官网截至测试时无当日文章）。合计新增19篇，URL唯一19，正文可用19，最短1,562字符。</x:v>
+        <x:v>验证通过：08-01 idle 0；08-02 idle 0；08-03 13；08-04 6；08-05 0（官网截至测试时无当日文章）。合计新增19篇，URL唯一19，正文可用19，最短1,562字符。
+19条候选正文均为full；新增4条、重复跳过15条，未覆盖远端既有记录。08-03为13条、08-04为6条。</x:v>
       </x:c>
       <x:c r="Z15" s="70" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>2026-08-06</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="38" customHeight="1">
@@ -5945,7 +5950,7 @@
         <x:v>2026-08-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="132" customHeight="1">
+    <x:row r="23" ht="186" customHeight="1">
       <x:c r="A23" s="82" t="n">
         <x:v>22</x:v>
       </x:c>
@@ -6016,13 +6021,15 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="X23" s="70" t="str">
-        <x:v>新增 RIOnews 下载、按日拆分及中国能源网专用导入器；接入 daily-news 与 channel-recovery 工作流；正式回补 2026-07-27—2026-08-04。</x:v>
+        <x:v>新增 RIOnews 下载、按日拆分及中国能源网专用导入器；接入 daily-news 与 channel-recovery 工作流；正式回补 2026-07-27—2026-08-04。
+2026-08-06 RIOnews历史数据合并：08-03发布24条、08-04发布5条，按规范化URL去重并新增。</x:v>
       </x:c>
       <x:c r="Y23" s="70" t="str">
-        <x:v>验证通过：07-28 22篇、08-03 24篇、08-04 5篇；合计51篇，URL唯一51，正文可用50篇，1篇短正文；08-04运行状态 healthy。</x:v>
+        <x:v>验证通过：07-28 22篇、08-03 24篇、08-04 5篇；合计51篇，URL唯一51，正文可用50篇，1篇短正文；08-04运行状态 healthy。
+新增29条、重复0条；正文184—11,614字，29条均为full。</x:v>
       </x:c>
       <x:c r="Z23" s="70" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>2026-08-06</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="38" customHeight="1">
@@ -6239,7 +6246,7 @@
         <x:v>2026-08-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="132" customHeight="1">
+    <x:row r="27" ht="186" customHeight="1">
       <x:c r="A27" s="82" t="n">
         <x:v>26</x:v>
       </x:c>
@@ -6308,16 +6315,18 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="X27" s="70" t="str">
-        <x:v>新增 国际能源网 RIOnews 媒体前缀映射；复用 API 下载、按日拆分与统一入库流程；正式回补 2026-07-27—2026-08-04。</x:v>
+        <x:v>新增 国际能源网 RIOnews 媒体前缀映射；复用 API 下载、按日拆分与统一入库流程；正式回补 2026-07-27—2026-08-04。
+2026-08-06 RIOnews历史数据合并：08-04发布记录5条按规范化URL去重并新增。</x:v>
       </x:c>
       <x:c r="Y27" s="70" t="str">
-        <x:v>验证通过：07-28 6篇、07-29 5篇、07-30 2篇、07-31 6篇、08-04 5篇，合计24篇；URL唯一24，正文可用24篇；08-04运行状态 healthy。</x:v>
+        <x:v>验证通过：07-28 6篇、07-29 5篇、07-30 2篇、07-31 6篇、08-04 5篇，合计24篇；URL唯一24，正文可用24篇；08-04运行状态 healthy。
+新增5条、重复0条；正文2,808—9,265字，5条均为full。</x:v>
       </x:c>
       <x:c r="Z27" s="70" t="str">
-        <x:v>2026-08-05</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="132" customHeight="1">
+        <x:v>2026-08-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="186" customHeight="1">
       <x:c r="A28" s="82" t="n">
         <x:v>27</x:v>
       </x:c>
@@ -6386,16 +6395,18 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="X28" s="70" t="str">
-        <x:v>新增 我爱电车网 RIOnews 媒体前缀映射；复用 API 下载、按日拆分与统一入库流程；正式回补 2026-07-27—2026-08-04。</x:v>
+        <x:v>新增 我爱电车网 RIOnews 媒体前缀映射；复用 API 下载、按日拆分与统一入库流程；正式回补 2026-07-27—2026-08-04。
+2026-08-06 RIOnews历史数据合并：08-03发布1条、08-04发布4条，按规范化URL去重并新增。</x:v>
       </x:c>
       <x:c r="Y28" s="70" t="str">
-        <x:v>验证通过：07-28 2篇、08-03 1篇、08-04 4篇，合计7篇；URL唯一7，正文可用7篇；08-04运行状态 healthy。</x:v>
+        <x:v>验证通过：07-28 2篇、08-03 1篇、08-04 4篇，合计7篇；URL唯一7，正文可用7篇；08-04运行状态 healthy。
+新增5条、重复0条；正文577—1,101字，5条均为full。</x:v>
       </x:c>
       <x:c r="Z28" s="70" t="str">
-        <x:v>2026-08-05</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="132" customHeight="1">
+        <x:v>2026-08-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="186" customHeight="1">
       <x:c r="A29" s="82" t="n">
         <x:v>28</x:v>
       </x:c>
@@ -6466,13 +6477,15 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="X29" s="70" t="str">
-        <x:v>新增 电池网 RIOnews 媒体前缀映射；复用 API 下载、按日拆分与统一入库流程；正式回补 2026-07-27—2026-08-04。</x:v>
+        <x:v>新增 电池网 RIOnews 媒体前缀映射；复用 API 下载、按日拆分与统一入库流程；正式回补 2026-07-27—2026-08-04。
+2026-08-06 RIOnews历史数据合并：08-04发布记录4条按规范化URL去重并新增。</x:v>
       </x:c>
       <x:c r="Y29" s="70" t="str">
-        <x:v>验证通过：07-27 1篇、08-04 4篇，合计5篇；URL唯一5，正文可用5篇；08-04运行状态 healthy。</x:v>
+        <x:v>验证通过：07-27 1篇、08-04 4篇，合计5篇；URL唯一5，正文可用5篇；08-04运行状态 healthy。
+新增4条、重复0条；正文1,078—2,665字，4条均为full。</x:v>
       </x:c>
       <x:c r="Z29" s="70" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>2026-08-06</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="38" customHeight="1">
@@ -6823,7 +6836,7 @@
         <x:v>2026-08-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="132" customHeight="1">
+    <x:row r="35" ht="186" customHeight="1">
       <x:c r="A35" s="82" t="n">
         <x:v>34</x:v>
       </x:c>
@@ -6894,13 +6907,15 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="X35" s="70" t="str">
-        <x:v>新增 BatteriesNewsScraper；禁用自动 RSS 发现，确保只抓 Latest；新增模块边界、Load More 分页、日期截断、URL 去重和正文边界测试。</x:v>
+        <x:v>新增 BatteriesNewsScraper；禁用自动 RSS 发现，确保只抓 Latest；新增模块边界、Load More 分页、日期截断、URL 去重和正文边界测试。
+2026-08-06 历史数据合并：08-04发布记录1条按规范化URL去重并新增，重新生成对应CSV。</x:v>
       </x:c>
       <x:c r="Y35" s="70" t="str">
-        <x:v>实站验证：Latest 首屏29个候选，Load More=/page/2/；08-04命中1篇，正文898字，crawl_mode=listing，状态 healthy。</x:v>
+        <x:v>实站验证：Latest 首屏29个候选，Load More=/page/2/；08-04命中1篇，正文898字，crawl_mode=listing，状态 healthy。
+新增1条、重复0条；正文1,359字且完整性状态为full。</x:v>
       </x:c>
       <x:c r="Z35" s="70" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>2026-08-06</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="38" customHeight="1">
@@ -9651,7 +9666,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c7716e04cb349a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcedd7bab35444b20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add Data Center Knowledge channel
</commit_message>
<xml_diff>
--- a/channel-maintenance-pv-fixed.xlsx
+++ b/channel-maintenance-pv-fixed.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="Rb14bb4c440164193"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="定义与优先级" sheetId="2" r:id="Rb90fe51ca2bb429e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题清单" sheetId="3" r:id="Ra313d2d4024c49d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周采集明细" sheetId="4" r:id="R09efb064357149b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="渠道维护总表" sheetId="5" r:id="R138856ad05704577"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R7461829629ac4e4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="定义与优先级" sheetId="2" r:id="R7e6f706d132b4843"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题清单" sheetId="3" r:id="Rb5717aa7a8d04120"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="周采集明细" sheetId="4" r:id="R8ae9a67096cc487f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="渠道维护总表" sheetId="5" r:id="Rf154138074ee4259"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -908,22 +908,22 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="51" t="n">
-        <x:f>COUNTA('渠道维护总表'!$B$2:$B$58)</x:f>
-        <x:v>57</x:v>
+        <x:f>COUNTA('渠道维护总表'!$B$2:$B$59)</x:f>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B9" s="52"/>
       <x:c r="C9" s="52" t="n">
-        <x:f>COUNTIF('渠道维护总表'!$F$2:$F$58,"零产出异常")+COUNTIF('渠道维护总表'!$F$2:$F$58,"正文质量降级")</x:f>
+        <x:f>COUNTIF('渠道维护总表'!$F$2:$F$59,"零产出异常")+COUNTIF('渠道维护总表'!$F$2:$F$59,"正文质量降级")</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D9" s="52"/>
       <x:c r="E9" s="52" t="n">
-        <x:f>SUM('渠道维护总表'!$L$2:$L$58)</x:f>
+        <x:f>SUM('渠道维护总表'!$L$2:$L$59)</x:f>
         <x:v>83</x:v>
       </x:c>
       <x:c r="F9" s="52"/>
       <x:c r="G9" s="52" t="n">
-        <x:f>COUNTIF('渠道维护总表'!$F$2:$F$58,"已配置跳过")</x:f>
+        <x:f>COUNTIF('渠道维护总表'!$F$2:$F$59,"已配置跳过")</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="H9" s="54"/>
@@ -3827,7 +3827,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8231e6c89bc7439f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R982449afb69b4f58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4298,7 +4298,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R009bad2da34f4077"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re22df8520f8c4b1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8477,32 +8477,84 @@
       </x:c>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="82"/>
-      <x:c r="B59" s="82"/>
-      <x:c r="C59" s="82"/>
-      <x:c r="D59" s="82"/>
-      <x:c r="E59" s="70"/>
-      <x:c r="F59" s="82"/>
-      <x:c r="G59" s="82"/>
-      <x:c r="H59" s="82"/>
-      <x:c r="I59" s="82"/>
-      <x:c r="J59" s="82"/>
-      <x:c r="K59" s="82"/>
-      <x:c r="L59" s="82"/>
-      <x:c r="M59" s="82"/>
-      <x:c r="N59" s="82"/>
-      <x:c r="O59" s="82"/>
-      <x:c r="P59" s="82"/>
-      <x:c r="Q59" s="82"/>
-      <x:c r="R59" s="82"/>
-      <x:c r="S59" s="70"/>
-      <x:c r="T59" s="70"/>
-      <x:c r="U59" s="83"/>
-      <x:c r="V59" s="83"/>
-      <x:c r="W59" s="70"/>
-      <x:c r="X59" s="70"/>
-      <x:c r="Y59" s="70"/>
-      <x:c r="Z59" s="82"/>
+      <x:c r="A59" s="82" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B59" s="82" t="str">
+        <x:v>Data Center Knowledge</x:v>
+      </x:c>
+      <x:c r="C59" s="82" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D59" s="82" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="E59" s="70" t="str">
+        <x:v>https://www.datacenterknowledge.com/latest-news</x:v>
+      </x:c>
+      <x:c r="F59" s="82" t="str">
+        <x:v>健康</x:v>
+      </x:c>
+      <x:c r="G59" s="82" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H59" s="82" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I59" s="82" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J59" s="82" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K59" s="82" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L59" s="82" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M59" s="82" t="str">
+        <x:v>2026-08-06</x:v>
+      </x:c>
+      <x:c r="N59" s="82" t="str">
+        <x:v>listing+rss</x:v>
+      </x:c>
+      <x:c r="O59" s="82" t="n">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="P59" s="82" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q59" s="82" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R59" s="82" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S59" s="70" t="str">
+        <x:v>ADD-002</x:v>
+      </x:c>
+      <x:c r="T59" s="70" t="str">
+        <x:v>新增每日抓取渠道；官方 RSS 仅含 description 摘要，且 RSS 可能早于 Latest News 列表刷新。</x:v>
+      </x:c>
+      <x:c r="U59" s="83" t="str">
+        <x:v>用户要求同时覆盖顶部新闻、下方列表及翻页，并判断 RSS 是否有全文。</x:v>
+      </x:c>
+      <x:c r="V59" s="83" t="str">
+        <x:v>RSS 与 Latest News 多区块候选取并集，按 URL 去重、Next 翻页、详情页取全文；RSS 独有链接也纳入，避免列表延迟漏抓。</x:v>
+      </x:c>
+      <x:c r="W59" s="70" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="X59" s="70" t="str">
+        <x:v>新增 DataCenterKnowledgeScraper 与注册；设定 .ArticleBase-BodyContent_Article 全文边界；补充列表合并、去重、翻页、RSS 先发和摘要降级测试。</x:v>
+      </x:c>
+      <x:c r="Y59" s="70" t="str">
+        <x:v>2026-08-06 在线试抓：95 个去重候选，命中 1 篇当日文章，详情页严格正文 4,264 字符，content_status=full，无作者、推荐、侧栏或页脚噪声。</x:v>
+      </x:c>
+      <x:c r="Z59" s="82" t="str">
+        <x:v>2026-08-06</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="82"/>
@@ -9666,7 +9718,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcedd7bab35444b20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03c356d3831b4d4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>